<commit_message>
tracking update 28.06.2026 15:00
</commit_message>
<xml_diff>
--- a/files/UAE_007_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_22.06.2026.xlsx
+++ b/files/UAE_007_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_22.06.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#7\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#7_APMG_STPARTSmix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F017AB2E-D26D-4976-9299-5C49E8181924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EAD91E8-7042-4926-B3E8-51508746B60B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1155" yWindow="2340" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="540" yWindow="1710" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э7" sheetId="1" r:id="rId1"/>
@@ -397,7 +397,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
@@ -570,12 +570,6 @@
     </xf>
     <xf numFmtId="10" fontId="12" fillId="8" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2005,15 +1999,15 @@
         <v>2711.5156740340813</v>
       </c>
       <c r="V2" s="31">
-        <v>3600</v>
+        <v>3675</v>
       </c>
       <c r="W2" s="32">
         <f>IFERROR((V2-U2)/U2,"")</f>
-        <v>0.32767073208323683</v>
+        <v>0.35533053900163758</v>
       </c>
       <c r="X2" s="33">
         <f t="shared" ref="X2:X7" si="9">V2*E2</f>
-        <v>13363200</v>
+        <v>13641600</v>
       </c>
       <c r="Y2" s="33">
         <f t="shared" ref="Y2:Y7" si="10">IFERROR(U2*E2,"")</f>
@@ -8469,7 +8463,7 @@
       <c r="J8" s="51"/>
       <c r="K8" s="51"/>
       <c r="L8" s="51"/>
-      <c r="M8" s="63"/>
+      <c r="M8" s="58"/>
       <c r="N8" s="48"/>
       <c r="O8" s="52"/>
       <c r="P8" s="52"/>
@@ -8478,7 +8472,7 @@
       <c r="S8" s="52"/>
       <c r="T8" s="52"/>
       <c r="U8" s="53"/>
-      <c r="V8" s="64"/>
+      <c r="V8" s="58"/>
       <c r="W8" s="54"/>
       <c r="X8" s="55"/>
       <c r="Y8" s="55"/>
@@ -9506,7 +9500,7 @@
       <c r="W9" s="54"/>
       <c r="X9" s="55">
         <f>SUM(X2:X7)</f>
-        <v>22451220</v>
+        <v>22729620</v>
       </c>
       <c r="Y9" s="55">
         <f>SUM(Y2:Y7)</f>
@@ -9629,7 +9623,7 @@
       </c>
       <c r="Y12" s="62">
         <f>(X9-Y9)/Y9</f>
-        <v>0.34258323754507514</v>
+        <v>0.35923156103629517</v>
       </c>
     </row>
     <row r="13" spans="1:1022" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
tracking update 29.06.2026 17:42
</commit_message>
<xml_diff>
--- a/files/UAE_007_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_22.06.2026.xlsx
+++ b/files/UAE_007_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_22.06.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#7_APMG_STPARTSmix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EAD91E8-7042-4926-B3E8-51508746B60B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0CF6F3-E04A-41F6-88FB-31CC258C9985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="540" yWindow="1710" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2010" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э7" sheetId="1" r:id="rId1"/>

</xml_diff>